<commit_message>
fixes units form redd metadata, generates and validates xml
</commit_message>
<xml_diff>
--- a/data-raw/metadata/battle_redd_metadata.xlsx
+++ b/data-raw/metadata/battle_redd_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-battle-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D12AB954-9F7E-4AB2-8010-A29E8254DE60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E590AD-E85B-42A2-9DFA-E01E48D0F1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5310" yWindow="1150" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="62">
   <si>
     <t xml:space="preserve">attribute_name </t>
   </si>
@@ -101,9 +101,6 @@
   </si>
   <si>
     <t>feetPerSecond</t>
-  </si>
-  <si>
-    <t>meter</t>
   </si>
   <si>
     <t>redd</t>
@@ -628,13 +625,13 @@
         <v>21</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" s="13" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E2" s="13" t="s">
         <v>17</v>
@@ -644,14 +641,14 @@
       <c r="H2" s="15"/>
       <c r="I2" s="14"/>
       <c r="J2" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K2" s="14"/>
       <c r="L2" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M2" s="16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
@@ -669,16 +666,16 @@
     </row>
     <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E3" s="13" t="s">
         <v>14</v>
@@ -707,16 +704,16 @@
     </row>
     <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>14</v>
@@ -745,16 +742,16 @@
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>14</v>
@@ -783,16 +780,16 @@
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>16</v>
@@ -801,10 +798,10 @@
         <v>15</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I6" s="14"/>
       <c r="J6" s="15"/>
@@ -831,16 +828,16 @@
     </row>
     <row r="7" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" s="13" t="s">
         <v>14</v>
@@ -869,16 +866,16 @@
     </row>
     <row r="8" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E8" s="13" t="s">
         <v>14</v>
@@ -907,16 +904,16 @@
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E9" s="13" t="s">
         <v>16</v>
@@ -925,10 +922,10 @@
         <v>15</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I9" s="14"/>
       <c r="J9" s="15"/>
@@ -955,16 +952,16 @@
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>15</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>16</v>
@@ -973,10 +970,10 @@
         <v>15</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I10" s="14"/>
       <c r="J10" s="15"/>
@@ -1003,16 +1000,16 @@
     </row>
     <row r="11" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>15</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E11" s="13" t="s">
         <v>16</v>
@@ -1021,10 +1018,10 @@
         <v>15</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I11" s="14"/>
       <c r="J11" s="15"/>
@@ -1051,16 +1048,16 @@
     </row>
     <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>15</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E12" s="13" t="s">
         <v>16</v>
@@ -1069,10 +1066,10 @@
         <v>15</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I12" s="14"/>
       <c r="J12" s="15"/>
@@ -1099,16 +1096,16 @@
     </row>
     <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>15</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E13" s="13" t="s">
         <v>16</v>
@@ -1117,10 +1114,10 @@
         <v>15</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I13" s="14"/>
       <c r="J13" s="15"/>
@@ -1147,16 +1144,16 @@
     </row>
     <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E14" s="13" t="s">
         <v>14</v>
@@ -1185,16 +1182,16 @@
     </row>
     <row r="15" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E15" s="13" t="s">
         <v>14</v>
@@ -1223,16 +1220,16 @@
     </row>
     <row r="16" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E16" s="13" t="s">
         <v>14</v>
@@ -1270,7 +1267,7 @@
         <v>15</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>16</v>
@@ -1282,7 +1279,7 @@
         <v>24</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I17" s="14"/>
       <c r="J17" s="15"/>

</xml_diff>